<commit_message>
Implementacion del dashboard, ETL pipeline, persistencia Firebase y scheduler
</commit_message>
<xml_diff>
--- a/data/test/cronograma_prueba.xlsx
+++ b/data/test/cronograma_prueba.xlsx
@@ -491,12 +491,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -549,12 +549,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>19/02/2025</t>
+          <t>01/04/2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>19/02/2025</t>
+          <t>01/04/2025</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>29/04/2025</t>
+          <t>09/06/2025</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>29/04/2025</t>
+          <t>09/06/2025</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -723,12 +723,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -781,12 +781,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -835,12 +835,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17/05/2025</t>
+          <t>27/06/2025</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17/05/2025</t>
+          <t>27/06/2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>07/03/2025</t>
+          <t>17/04/2025</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07/03/2025</t>
+          <t>17/04/2025</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -951,12 +951,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1067,12 +1067,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>05/05/2025</t>
+          <t>15/06/2025</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05/05/2025</t>
+          <t>15/06/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1125,12 +1125,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15/05/2025</t>
+          <t>25/06/2025</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>15/05/2025</t>
+          <t>25/06/2025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1179,12 +1179,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1237,12 +1237,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>31/03/2025</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>31/03/2025</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1291,12 +1291,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>09/04/2025</t>
+          <t>20/05/2025</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>09/04/2025</t>
+          <t>20/05/2025</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1407,12 +1407,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>19/01/2025</t>
+          <t>01/03/2025</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>19/01/2025</t>
+          <t>01/03/2025</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>13/02/2025</t>
+          <t>26/03/2025</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>13/02/2025</t>
+          <t>26/03/2025</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1581,12 +1581,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>25/03/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>25/03/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1639,12 +1639,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>16/05/2025</t>
+          <t>26/06/2025</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>16/05/2025</t>
+          <t>26/06/2025</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1693,12 +1693,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>19/05/2025</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>19/05/2025</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1747,12 +1747,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>21/04/2025</t>
+          <t>01/06/2025</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>21/04/2025</t>
+          <t>01/06/2025</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1805,12 +1805,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1921,12 +1921,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>06/06/2025</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>06/06/2025</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1979,12 +1979,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2037,12 +2037,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>19/05/2025</t>
+          <t>29/06/2025</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>19/05/2025</t>
+          <t>29/06/2025</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2095,12 +2095,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>26/03/2025</t>
+          <t>06/05/2025</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>26/03/2025</t>
+          <t>06/05/2025</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2149,12 +2149,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10/05/2025</t>
+          <t>20/06/2025</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10/05/2025</t>
+          <t>20/06/2025</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2207,12 +2207,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16/05/2025</t>
+          <t>26/06/2025</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>16/05/2025</t>
+          <t>26/06/2025</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2265,12 +2265,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>06/06/2025</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>06/06/2025</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2319,12 +2319,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2373,12 +2373,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>24/04/2025</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>24/04/2025</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2431,12 +2431,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>19/05/2025</t>
+          <t>29/06/2025</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>19/05/2025</t>
+          <t>29/06/2025</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2489,12 +2489,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>18/05/2025</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>18/05/2025</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2547,12 +2547,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>10/06/2025</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>10/06/2025</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2605,12 +2605,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2663,12 +2663,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16/05/2025</t>
+          <t>26/06/2025</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>16/05/2025</t>
+          <t>26/06/2025</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2721,12 +2721,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>18/05/2025</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>18/05/2025</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2779,12 +2779,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>18/03/2025</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>18/03/2025</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2837,12 +2837,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>20/03/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>20/03/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2891,12 +2891,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">

</xml_diff>